<commit_message>
add Masters column to indicate Masters presentation order
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/registration/Registration.xlsx
+++ b/owlcms/src/main/resources/templates/registration/Registration.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamyj\git\owlcms4\owlcms\src\main\resources\templates\registration\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78CCCC79-8904-42FB-A76C-B13E8C3C3BC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF35E24B-CCD6-4BB4-ADD1-34A0A85C544F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-25890" yWindow="6615" windowWidth="25215" windowHeight="7455" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Athletes" sheetId="1" r:id="rId1"/>
@@ -104,7 +104,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="67">
   <si>
     <t>M/F</t>
   </si>
@@ -299,6 +299,12 @@
   </si>
   <si>
     <t>${l.group}</t>
+  </si>
+  <si>
+    <t>${t.get("Masters")}</t>
+  </si>
+  <si>
+    <t>${g.masters}</t>
   </si>
 </sst>
 </file>
@@ -874,23 +880,7 @@
     <cellStyle name="Title" xfId="33" builtinId="15" customBuiltin="1"/>
     <cellStyle name="Total" xfId="34" builtinId="25" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="4">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="34"/>
-          <bgColor indexed="13"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="34"/>
-          <bgColor indexed="13"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -21129,22 +21119,12 @@
   </sheetData>
   <sheetProtection insertRows="0"/>
   <phoneticPr fontId="2" type="noConversion"/>
-  <conditionalFormatting sqref="B3:E3">
-    <cfRule type="expression" dxfId="3" priority="6" stopIfTrue="1">
-      <formula>AND((#REF!),#REF!,#REF!)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B5:E1800">
-    <cfRule type="expression" dxfId="2" priority="2" stopIfTrue="1">
-      <formula>AND((#REF!),#REF!,#REF!)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F3">
+  <conditionalFormatting sqref="B3:F3">
     <cfRule type="expression" dxfId="1" priority="5" stopIfTrue="1">
       <formula>AND((#REF!),#REF!,#REF!)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F5:F1800">
+  <conditionalFormatting sqref="B5:F1800">
     <cfRule type="expression" dxfId="0" priority="1" stopIfTrue="1">
       <formula>AND((#REF!),#REF!,#REF!)</formula>
     </cfRule>
@@ -21157,7 +21137,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:V5"/>
+  <dimension ref="A1:W5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="25.42578125" customWidth="1"/>
@@ -21165,7 +21145,7 @@
     <col min="6" max="21" width="12.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
         <v>9</v>
       </c>
@@ -21174,7 +21154,7 @@
       <c r="D1" s="21"/>
       <c r="E1" s="21"/>
     </row>
-    <row r="2" spans="1:22" s="11" customFormat="1" ht="48.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23" s="11" customFormat="1" ht="48.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
         <v>1</v>
       </c>
@@ -21241,8 +21221,11 @@
       <c r="V2" s="11" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W2" s="11" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>19</v>
       </c>
@@ -21250,8 +21233,11 @@
       <c r="E3" s="1"/>
       <c r="I3" s="5"/>
       <c r="J3" s="5"/>
-    </row>
-    <row r="4" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="W3" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>20</v>
       </c>
@@ -21319,7 +21305,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
fix registration file import; closes #1278
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/registration/Registration.xlsx
+++ b/owlcms/src/main/resources/templates/registration/Registration.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamyj\git\owlcms4\owlcms\src\main\resources\templates\registration\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32948985-0486-495B-8152-9126E10BD82F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AC98B7A-1B20-4B87-8B01-51AADEF584EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2565" yWindow="2895" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Athletes" sheetId="1" r:id="rId1"/>
@@ -301,9 +301,6 @@
     <t>${l.group}</t>
   </si>
   <si>
-    <t>${t.get("Masters")}</t>
-  </si>
-  <si>
     <t>${g.masters}</t>
   </si>
   <si>
@@ -311,6 +308,9 @@
   </si>
   <si>
     <t>${g.reserveJury}</t>
+  </si>
+  <si>
+    <t>${t.get("Competition.masters")}</t>
   </si>
 </sst>
 </file>
@@ -21228,10 +21228,10 @@
         <v>49</v>
       </c>
       <c r="W2" s="11" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="X2" s="11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.25">
@@ -21311,10 +21311,10 @@
         <v>34</v>
       </c>
       <c r="W4" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="X4" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
added doctor, fixed range
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/registration/Registration.xlsx
+++ b/owlcms/src/main/resources/templates/registration/Registration.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamyj\git\owlcms4\owlcms\src\main\resources\templates\registration\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\git\owlcms_v23\owlcms\src\main\resources\templates\registration\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AC98B7A-1B20-4B87-8B01-51AADEF584EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F63DEB94-E40A-4D6B-B9E5-50DBFE842656}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2565" yWindow="2895" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Athletes" sheetId="1" r:id="rId1"/>
@@ -104,7 +104,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="71">
   <si>
     <t>M/F</t>
   </si>
@@ -311,6 +311,12 @@
   </si>
   <si>
     <t>${t.get("Competition.masters")}</t>
+  </si>
+  <si>
+    <t>${t.get("Doctor")}</t>
+  </si>
+  <si>
+    <t>${g.doctor}</t>
   </si>
 </sst>
 </file>
@@ -21143,7 +21149,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:X5"/>
+  <dimension ref="A1:Y5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="25.42578125" customWidth="1"/>
@@ -21151,7 +21157,7 @@
     <col min="6" max="21" width="12.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
         <v>9</v>
       </c>
@@ -21160,7 +21166,7 @@
       <c r="D1" s="21"/>
       <c r="E1" s="21"/>
     </row>
-    <row r="2" spans="1:24" s="11" customFormat="1" ht="48.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:25" s="11" customFormat="1" ht="48.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
         <v>1</v>
       </c>
@@ -21233,8 +21239,11 @@
       <c r="X2" s="11" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y2" s="11" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>19</v>
       </c>
@@ -21243,7 +21252,7 @@
       <c r="I3" s="5"/>
       <c r="J3" s="5"/>
     </row>
-    <row r="4" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>20</v>
       </c>
@@ -21316,8 +21325,11 @@
       <c r="X4" s="1" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Y4" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Add missing session import fields
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/registration/Registration.xlsx
+++ b/owlcms/src/main/resources/templates/registration/Registration.xlsx
@@ -104,7 +104,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="81">
   <si>
     <t>M/F</t>
   </si>
@@ -317,6 +317,36 @@
   </si>
   <si>
     <t>${g.doctor}</t>
+  </si>
+  <si>
+    <t>${t.get("TechnicalController3")}</t>
+  </si>
+  <si>
+    <t>${g.technicalController3}</t>
+  </si>
+  <si>
+    <t>${t.get("AccreditationRole.COMPETITION_DIRECTOR")}</t>
+  </si>
+  <si>
+    <t>${g.competitionDirector}</t>
+  </si>
+  <si>
+    <t>${t.get("TIS1")}</t>
+  </si>
+  <si>
+    <t>${g.tis1}</t>
+  </si>
+  <si>
+    <t>${t.get("TIS2")}</t>
+  </si>
+  <si>
+    <t>${g.tis2}</t>
+  </si>
+  <si>
+    <t>${t.get("CJ_BreakDuration")}</t>
+  </si>
+  <si>
+    <t>${g.cleanJerkBreakDuration}</t>
   </si>
 </sst>
 </file>
@@ -21148,16 +21178,16 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:Y5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:AD5"/>
+  <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="25.42578125" customWidth="1"/>
     <col min="4" max="5" width="16.42578125" style="5" customWidth="1"/>
     <col min="6" max="21" width="12.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" ht="37.5" customHeight="1" ns3:dyDescent="0.25">
       <c r="A1" s="21" t="s">
         <v>9</v>
       </c>
@@ -21166,7 +21196,7 @@
       <c r="D1" s="21"/>
       <c r="E1" s="21"/>
     </row>
-    <row r="2" spans="1:25" s="11" customFormat="1" ht="48.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" s="11" customFormat="1" ht="48.6" customHeight="1" ns3:dyDescent="0.25">
       <c r="A2" s="11" t="s">
         <v>1</v>
       </c>
@@ -21206,44 +21236,59 @@
       <c r="M2" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="N2" s="11" t="s">
+      <c r="N2" t="s" s="11">
+        <v>71</v>
+      </c>
+      <c r="O2" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="O2" s="11" t="s">
+      <c r="P2" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="P2" s="11" t="s">
+      <c r="Q2" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="Q2" s="11" t="s">
+      <c r="R2" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="R2" s="11" t="s">
+      <c r="S2" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="S2" s="11" t="s">
+      <c r="T2" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="T2" s="11" t="s">
+      <c r="U2" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="U2" s="11" t="s">
+      <c r="V2" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="V2" s="11" t="s">
+      <c r="W2" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="W2" s="11" t="s">
+      <c r="X2" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="X2" s="11" t="s">
+      <c r="Y2" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="Y2" s="11" t="s">
+      <c r="Z2" s="11" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="AA2" t="s" s="11">
+        <v>73</v>
+      </c>
+      <c r="AB2" t="s" s="11">
+        <v>75</v>
+      </c>
+      <c r="AC2" t="s" s="11">
+        <v>77</v>
+      </c>
+      <c r="AD2" t="s" s="11">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="3" spans="1:30" ns3:dyDescent="0.25">
       <c r="A3" t="s">
         <v>19</v>
       </c>
@@ -21252,7 +21297,7 @@
       <c r="I3" s="5"/>
       <c r="J3" s="5"/>
     </row>
-    <row r="4" spans="1:25" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:30" s="1" customFormat="1" ns3:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>20</v>
       </c>
@@ -21292,44 +21337,59 @@
       <c r="M4" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="N4" s="1" t="s">
+      <c r="N4" t="s" s="1">
+        <v>72</v>
+      </c>
+      <c r="O4" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="O4" s="1" t="s">
+      <c r="P4" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="P4" s="1" t="s">
+      <c r="Q4" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="Q4" s="1" t="s">
+      <c r="R4" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="R4" s="1" t="s">
+      <c r="S4" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="S4" s="1" t="s">
+      <c r="T4" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="T4" s="1" t="s">
+      <c r="U4" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="U4" s="1" t="s">
+      <c r="V4" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="V4" s="1" t="s">
+      <c r="W4" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="W4" s="1" t="s">
+      <c r="X4" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="X4" s="1" t="s">
+      <c r="Y4" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="Y4" s="1" t="s">
+      <c r="Z4" s="1" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="AA4" t="s" s="1">
+        <v>74</v>
+      </c>
+      <c r="AB4" t="s" s="1">
+        <v>76</v>
+      </c>
+      <c r="AC4" t="s" s="1">
+        <v>78</v>
+      </c>
+      <c r="AD4" t="s" s="1">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="5" spans="1:30" ns3:dyDescent="0.25">
       <c r="A5" t="s">
         <v>10</v>
       </c>

</xml_diff>